<commit_message>
feat(F-NAR-016): TREE-DIF-049 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-049.xlsx
+++ b/stories/arbres/TREE-DIF-049.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dehors, la mare a trop de vent. Le salon est tiède, tout calme. Le tapis sent encore le savon. Les manteaux sèchent, près du radiateur. Le seau bleu est vide, Sarah. Des ciseaux brillent sur la table. Je fais un étang, pour Nino. Tu lui proposes, tout calme ? Oui, papa. En ce moment, Sarah coupe un poisson. Le papier jaune craque, tout doux. Merci, tu tiens le seau bien.</t>
+          <t>Dehors, la mare a trop de vent. Le salon est tiède, tout calme. Le tapis sent encore le savon. Les manteaux sèchent, près du radiateur. Le seau bleu est vide, Sarah. Des ciseaux brillent sur la table. Je fais une mare, pour Nino. Tu lui proposes, tout calme ? Oui, papa. En ce moment, Sarah coupe un poisson. Le papier jaune craque, tout doux. Merci, tu tiens le seau bien.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dehors, la mare a trop de vent. Le salon est tiède, tout calme. Le tapis sent encore le savon. Les manteaux sèchent, près du radiateur. Le seau bleu est vide, Sarah. Des ciseaux brillent sur la table. Je fais un étang, pour Nino. Tu lui proposes, tout calme ? Oui, papa. En ce moment, Sarah coupe un poisson. Le papier jaune craque, tout doux. Merci, tu tiens le seau bien.</t>
+          <t>Dehors, la mare a trop de vent. Le salon est tiède, tout calme. Le tapis sent encore le savon. Les manteaux sèchent, près du radiateur. Le seau bleu est vide, Sarah. Des ciseaux brillent sur la table. Je fais une mare, pour Nino. Tu lui proposes, tout calme ? Oui, papa. En ce moment, Sarah coupe un poisson. Le papier jaune craque, tout doux. Merci, tu tiens le seau bien.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1343,7 +1343,7 @@
 papa|Les manteaux sèchent, près du radiateur.
 maman|Le seau bleu est vide, Sarah.
 narrateur|Des ciseaux brillent sur la table.
-enfant-f|Je fais un étang, pour Nino.
+enfant-f|Je fais une mare, pour Nino.
 papa|Tu lui proposes, tout calme ?
 enfant-f|Oui, papa.
 narrateur|En ce moment, Sarah coupe un poisson.
@@ -2305,12 +2305,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sarah redescend du canapé, tout doux. Nino tourne la boîte, tout absorbé. Nino, la mare est prête. Il ne lève pas encore les yeux. Ma chanson n'est pas finie. Tu viens pêcher, d'en haut ? J'ai pas fini. Il écoute encore, tout concentré. Tu proposes comment, Sarah ?</t>
+          <t>Sarah redescend du canapé, tout doux. Nino tourne la petite clé, absorbé. Nino, la mare est prête. Une note tinte, encore la même. Elle n'a pas dit au revoir. On pêche après la note ? Cette chanson, d'abord. La boîte tient encore sa voix. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sarah redescend du canapé, tout doux. Nino tourne la boîte, tout absorbé. Nino, la mare est prête. Il ne lève pas encore les yeux. Ma chanson n'est pas finie. Tu viens pêcher, d'en haut ? J'ai pas fini. Il écoute encore, tout concentré. Tu proposes comment, Sarah ?</t>
+          <t>Sarah redescend du canapé, tout doux. Nino tourne la petite clé, absorbé. Nino, la mare est prête. Une note tinte, encore la même. Elle n'a pas dit au revoir. On pêche après la note ? Cette chanson, d'abord. La boîte tient encore sa voix. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2446,14 +2446,14 @@
       <c r="AW8" t="inlineStr">
         <is>
           <t>narrateur|Sarah redescend du canapé, tout doux.
-narrateur|Nino tourne la boîte, tout absorbé.
+narrateur|Nino tourne la petite clé, absorbé.
 enfant-f|Nino, la mare est prête.
-narrateur|Il ne lève pas encore les yeux.
-copain|Ma chanson n'est pas finie.
-enfant-f|Tu viens pêcher, d'en haut ?
-copain|J'ai pas fini.
-maman|Il écoute encore, tout concentré.
-papa|Tu proposes comment, Sarah ?</t>
+narrateur|Une note tinte, encore la même.
+copain|Elle n'a pas dit au revoir.
+enfant-f|On pêche après la note ?
+copain|Cette chanson, d'abord.
+maman|La boîte tient encore sa voix.
+papa|Tu restes près de lui ?</t>
         </is>
       </c>
     </row>
@@ -2672,12 +2672,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. La ficelle pend, sans bouger. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. La ficelle pend, sans bouger. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. La ficelle pend, sans bouger. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. La ficelle pend, sans bouger. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2812,15 +2812,15 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends un peu.
+          <t>enfant-f|J'attends la dernière note.
 copain|Merci, Sarah.
-narrateur|La boîte tourne sa dernière note.
+narrateur|Elle compte les tintes, sur ses doigts.
 narrateur|La ficelle pend, sans bouger.
-narrateur|Nino pose la clé, enfin.
-copain|Ma chanson est finie, maintenant.
+narrateur|La boîte s'arrête, pile.
+copain|Elle a dit au revoir.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé sa chanson finir.</t>
+copain|Oui, j'apporte la clé.
+papa|Tu as laissé la chanson finir.</t>
         </is>
       </c>
     </row>
@@ -2847,12 +2847,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. La ficelle garde encore un peu de savon. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. La ficelle garde encore un peu de savon. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. La ficelle garde encore un peu de savon. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. La ficelle garde encore un peu de savon. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2987,14 +2987,14 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Une nageoire jaune tremble dans le seau.
-copain|C'est une prise, Sarah ?
-enfant-f|Oui, elle est là.
-papa|Vous avez attendu le bon moment.
-maman|Le papier est encore un peu chaud.
+          <t>narrateur|La ficelle tremble, puis un papier vient.
+copain|Il a mordu, Sarah ?
+enfant-f|Oui, tout plat.
+papa|La chanson a laissé la place.
+maman|Le seau fait un petit ploc.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino souffle sur le poisson, tout petit.
-enfant-f|C'est notre mare, maintenant.
+narrateur|Nino pose la clé à côté du seau.
+enfant-f|La mare chante, maintenant.
 narrateur|Un peu de savon reste sur le papier.</t>
         </is>
       </c>
@@ -3022,12 +3022,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre le canapé. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre le canapé. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre le canapé. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre le canapé. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3162,15 +3162,15 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, je te propose la mare.
-narrateur|Elle parle tout contre le canapé.
+          <t>enfant-f|Nino, un poisson t'écoute.
+narrateur|Elle glisse un poisson contre le canapé.
 narrateur|Sa voix reste tout bas, près de lui.
-copain|J'ai entendu, Sarah.
-enfant-f|Tu peux dire non.
-copain|Oui, je viens.
-narrateur|Il ferme la boîte, tout doux.
-papa|Ta voix est restée tout bas.
-maman|Il a choisi de lui-même.</t>
+copain|Il a une oreille, lui aussi ?
+enfant-f|Oui, tout calme.
+copain|Je viens, alors.
+narrateur|Il pose la clé, sans la perdre.
+papa|Tu as parlé tout contre lui.
+maman|Il a dit oui, tout seul.</t>
         </is>
       </c>
     </row>
@@ -3197,12 +3197,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. La ficelle garde encore un peu de savon. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. La ficelle garde encore un peu de savon. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. La ficelle garde encore un peu de savon. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. La ficelle garde encore un peu de savon. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3337,14 +3337,14 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|La boîte est fermée, contre le genou.
-enfant-f|Tu as dit oui, tout bas.
-copain|J'avais entendu, près de toi.
-papa|Ta voix est restée tout bas.
-maman|Pêchez un peu, tout doux.
+          <t>narrateur|Le poisson collé écoute encore, un peu.
+enfant-f|Il t'a attendu, tout bas.
+copain|J'ai dit oui, près de toi.
+papa|Ta voix n'a pas cassé la note.
+maman|Pêchez, maintenant, tout doux.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino pose sa joue, tout calme.
-enfant-f|Reste autant que tu veux.
+narrateur|Nino tient le bâton, tout calme.
+enfant-f|On tire ensemble, tout lent.
 narrateur|La clé de la boîte dort, enfin.</t>
         </is>
       </c>
@@ -3372,12 +3372,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit au pied du canapé. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit au pied du canapé. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit au pied du canapé. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit au pied du canapé. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3515,12 +3515,12 @@
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit au pied du canapé.
 narrateur|Elle ne touche pas la clé.
-copain|Tu écoutes, toi aussi ?
-enfant-f|Oui, avec toi.
-narrateur|Deux oreilles, maintenant, sur la boîte.
-copain|Après, on va pêcher.
-papa|Tu es restée près de lui.
-maman|Il a proposé la suite.</t>
+copain|Tu entends le ding, toi aussi ?
+enfant-f|Oui, dans le ventre.
+narrateur|Un dernier ding les fait sauter.
+copain|On pêche, après ça.
+papa|Tu as écouté sa boîte.
+maman|C'est lui qui a dit après.</t>
         </is>
       </c>
     </row>
@@ -3547,12 +3547,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. La ficelle garde encore un peu de savon. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. La ficelle garde encore un peu de savon. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. La ficelle garde encore un peu de savon. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. La ficelle garde encore un peu de savon. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3687,14 +3687,14 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|Après la chanson, la ficelle descend.
-copain|On a écouté ensemble, d'abord.
-enfant-f|Puis tu as dit : on y va.
-maman|Deux oreilles, puis un poisson.
-papa|Le salon redevient calme.
+          <t>narrateur|Après le ding, la ficelle descend.
+copain|On a sauté, d'abord.
+enfant-f|Puis tu as dit : on pêche.
+maman|Un ding, puis un poisson.
+papa|Le salon redevient tiède.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino rit, tout petit.
-enfant-f|La mare t'a attendu.
+narrateur|Nino rit encore, tout petit.
+enfant-f|La mare a attendu le ding.
 narrateur|Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
@@ -3722,12 +3722,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Un camion jaune passe sous le canapé. Nino le pousse, tout concentré. Nino, on pêche d'en haut. Mon camion n'est pas garé. Tu viens sur le canapé ? Après, peut-être. Les roues font un petit rrr. Il conduit encore, tout calme. Tu proposes comment, Sarah ?</t>
+          <t>Un camion jaune passe sous le canapé. Nino le pousse entre deux livres. Nino, on pêche d'en haut. Il va au garage, encore. Tu viens sur le canapé ? Le garage, d'abord. Les roues font un petit rrr. Il range encore sa route. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Un camion jaune passe sous le canapé. Nino le pousse, tout concentré. Nino, on pêche d'en haut. Mon camion n'est pas garé. Tu viens sur le canapé ? Après, peut-être. Les roues font un petit rrr. Il conduit encore, tout calme. Tu proposes comment, Sarah ?</t>
+          <t>Un camion jaune passe sous le canapé. Nino le pousse entre deux livres. Nino, on pêche d'en haut. Il va au garage, encore. Tu viens sur le canapé ? Le garage, d'abord. Les roues font un petit rrr. Il range encore sa route. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3863,14 +3863,14 @@
       <c r="AW16" t="inlineStr">
         <is>
           <t>narrateur|Un camion jaune passe sous le canapé.
-narrateur|Nino le pousse, tout concentré.
+narrateur|Nino le pousse entre deux livres.
 enfant-f|Nino, on pêche d'en haut.
-copain|Mon camion n'est pas garé.
+copain|Il va au garage, encore.
 enfant-f|Tu viens sur le canapé ?
-copain|Après, peut-être.
+copain|Le garage, d'abord.
 narrateur|Les roues font un petit rrr.
-maman|Il conduit encore, tout calme.
-papa|Tu proposes comment, Sarah ?</t>
+maman|Il range encore sa route.
+papa|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -4089,12 +4089,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le canapé garde sa rive, encore. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le canapé garde sa rive, encore. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le canapé garde sa rive, encore. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le canapé garde sa rive, encore. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4229,15 +4229,15 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends qu'il gare.
+          <t>enfant-f|J'attends le garage.
 copain|Merci, Sarah.
 narrateur|Le canapé garde sa rive, encore.
-narrateur|Le camion s'arrête, pile.
-copain|C'est garé, maintenant.
+narrateur|Le camion se glisse entre deux livres.
+copain|Il est rentré, maintenant.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé son camion finir.
-maman|Il a dit oui, à son heure.</t>
+copain|Oui, je laisse les roues.
+papa|Tu as laissé le garage finir.
+maman|Il a dit oui, après.</t>
         </is>
       </c>
     </row>
@@ -4264,12 +4264,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. La ficelle garde encore un peu de savon. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. La ficelle garde encore un peu de savon. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. La ficelle garde encore un peu de savon. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. La ficelle garde encore un peu de savon. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4404,14 +4404,14 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|Le camion dort, près du seau.
-copain|J'ai fini, Sarah.
-enfant-f|Tu as dit oui.
-papa|Vous tenez tous les deux, maintenant.
-maman|Le poisson descend jusqu'à vous.
+          <t>narrateur|Le camion dort entre les livres.
+copain|Le garage est fermé, Sarah.
+enfant-f|Tu as dit oui, après.
+papa|Les roues se sont tues.
+maman|Le poisson glisse vers le seau.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino tape deux fois, tout doux.
-enfant-f|C'est le signal.
+narrateur|Nino souffle sur la nageoire, tout petit.
+enfant-f|Il nage, dans le bleu.
 narrateur|Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
@@ -4439,12 +4439,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sous le canapé. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur le capot. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sous le canapé. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur le capot. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4579,15 +4579,15 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un poisson dans le camion ?
-narrateur|Elle tend le poisson, sous le canapé.
-copain|Un tout petit, alors.
+          <t>enfant-f|Nino, un poisson voyageur ?
+narrateur|Elle pose le poisson sur le capot.
+copain|Il tient, sur le camion ?
+enfant-f|Tout plat, oui.
+narrateur|Le papier colle un peu, puis tient.
+copain|On va jusqu'au seau, alors.
 enfant-f|D'accord.
-narrateur|Le papier glisse, tout doux.
-copain|Il est tout plat, dedans.
-enfant-f|On est deux, maintenant.
-papa|Le poisson est resté dans sa main.
-maman|Il a pris ce qu'il voulait.</t>
+papa|Le poisson a pris la route.
+maman|Il a choisi le voyage.</t>
         </is>
       </c>
     </row>
@@ -4614,12 +4614,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. La ficelle garde encore un peu de savon. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. La ficelle garde encore un peu de savon. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. La ficelle garde encore un peu de savon. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. La ficelle garde encore un peu de savon. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4754,13 +4754,13 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le camion a un poisson, maintenant.
-enfant-f|Le tien, et le mien.
-copain|Il était plat, Sarah.
-papa|Vous avez partagé sans tout casser.
-maman|La mare, au fond, pour deux.
+          <t>narrateur|Le camion roule jusqu'au seau.
+enfant-f|Le voyageur descend, tout plat.
+copain|Il a tenu sur le capot.
+papa|Vous avez fait une route, ensemble.
+maman|Le seau devient un port, maintenant.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino souffle, puis Sarah souffle.
+narrateur|Nino pousse une dernière fois, tout doux.
 enfant-f|On reste encore un peu.
 narrateur|Un poisson plat dort sur le bois.</t>
         </is>
@@ -4789,12 +4789,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste au pied du canapé. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste au pied du canapé. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste au pied du canapé. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste au pied du canapé. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4931,13 +4931,13 @@
         <is>
           <t>copain|Pas de poisson, Sarah.
 enfant-f|D'accord.
-enfant-f|Je garde le seau, alors.
+enfant-f|Je pêche ici, alors.
 narrateur|Le seau reste au pied du canapé.
-narrateur|Elle pêche de son côté, tout calme.
-copain|Tu peux parler, d'ici.
-enfant-f|Je reste près de toi.
+narrateur|Un poisson se colle à sa chaussette.
+copain|Il t'a pêchée, toi !
+enfant-f|Je ris, d'à côté.
 papa|Tu as gardé ton seau.
-maman|Vous êtes encore ensemble.</t>
+maman|Le camion est resté à lui.</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. La ficelle garde encore un peu de savon. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. La ficelle garde encore un peu de savon. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. La ficelle garde encore un peu de savon. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. La ficelle garde encore un peu de savon. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5104,14 +5104,14 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|Deux jeux restent côte à côte.
-copain|Tu n'as pas pris mon camion.
+          <t>narrateur|Le camion reste à sa place.
+copain|Tu n'as pas pris mes roues.
 enfant-f|Tu avais dit non.
-papa|Son camion est resté à lui.
-maman|Vous vous parlez encore, d'ici.
+papa|Son garage est resté à lui.
+maman|La chaussette a eu un poisson.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino tend une roue, alors.
-enfant-f|Je la prends, d'à côté.
+narrateur|Nino rit, puis pousse encore.
+enfant-f|Je pêche, tu roules.
 narrateur|Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
@@ -5139,12 +5139,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Nino s'assoit au bord du tapis. J'ai un chausson, Sarah. On pêche d'en haut, après. Il cherche l'autre, sous le canapé. Tu viens sur le canapé ? Quand j'ai mes chaussons, d'abord. Il enfile encore, tout calme. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino s'assoit au bord du tapis. J'ai un pied froid, Sarah. On pêche d'en haut, après. Un chausson manque, sous le canapé. Tu viens sur le canapé ? L'autre chausson, d'abord. Il fouille encore, tout calme. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Nino s'assoit au bord du tapis. J'ai un chausson, Sarah. On pêche d'en haut, après. Il cherche l'autre, sous le canapé. Tu viens sur le canapé ? Quand j'ai mes chaussons, d'abord. Il enfile encore, tout calme. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino s'assoit au bord du tapis. J'ai un pied froid, Sarah. On pêche d'en haut, après. Un chausson manque, sous le canapé. Tu viens sur le canapé ? L'autre chausson, d'abord. Il fouille encore, tout calme. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5280,14 +5280,14 @@
       <c r="AW24" t="inlineStr">
         <is>
           <t>narrateur|Nino s'assoit au bord du tapis.
-copain|J'ai un chausson, Sarah.
+copain|J'ai un pied froid, Sarah.
 enfant-f|On pêche d'en haut, après.
-narrateur|Il cherche l'autre, sous le canapé.
+narrateur|Un chausson manque, sous le canapé.
 enfant-f|Tu viens sur le canapé ?
-copain|Quand j'ai mes chaussons, d'abord.
-papa|Il enfile encore, tout calme.
-maman|L'autre chausson n'est pas là.
-papa|Tu proposes comment, Sarah ?</t>
+copain|L'autre chausson, d'abord.
+papa|Il fouille encore, tout calme.
+maman|Le second n'est pas là.
+papa|Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
     </row>
@@ -5506,12 +5506,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche sous le canapé, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille sous le canapé, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche sous le canapé, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille sous le canapé, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5647,14 +5647,14 @@
       <c r="AW26" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle cherche sous le canapé, tout doux.
-narrateur|Le second chausson apparaît, enfin.
-copain|Tu l'as vu, toi aussi ?
-enfant-f|Oui, sous le bord.
+narrateur|Elle fouille sous le canapé, tout doux.
+narrateur|Un chausson chaud apparaît, enfin.
+copain|Il s'était caché !
+enfant-f|Près du bord, oui.
 narrateur|Deux pieds, maintenant, tout chauds.
-copain|Il était là !
-papa|Tu as aidé à son heure.
-maman|Vous l'avez eu, tous les deux.</t>
+copain|On peut pêcher, là.
+papa|Tu as cherché avec lui.
+maman|Le pied froid n'a plus froid.</t>
         </is>
       </c>
     </row>
@@ -5681,12 +5681,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. La ficelle garde encore un peu de savon. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. La ficelle garde encore un peu de savon. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. La ficelle garde encore un peu de savon. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. La ficelle garde encore un peu de savon. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5822,13 +5822,13 @@
       <c r="AW27" t="inlineStr">
         <is>
           <t>narrateur|Les deux chaussons sont chauds, enfin.
-copain|On l'a eu, ensemble.
-enfant-f|Puis la mare est arrivée.
-papa|Vous avez aidé à son heure.
+copain|Le pied froid n'a plus froid.
+enfant-f|On peut pêcher, là.
+papa|Vous avez cherché ensemble.
 maman|Le seau attend encore, tout doux.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino fait un signe vers le tapis.
-enfant-f|La mare t'a vu, une minute.
+narrateur|Nino s'allonge, le pied au chaud.
+enfant-f|La mare est tiède, pour deux.
 narrateur|Un fil jaune passe, tout loin.</t>
         </is>
       </c>
@@ -5856,12 +5856,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent la rive du canapé. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers la rive du canapé. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent la rive du canapé. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers la rive du canapé. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -5999,11 +5999,11 @@
           <t>enfant-f|Un tout petit regard, Nino ?
 copain|Très petit, alors.
 enfant-f|D'accord.
-narrateur|Ils regardent la rive du canapé.
+narrateur|Ils se penchent vers la rive du canapé.
 narrateur|Un poisson jaune brille, une seconde.
-copain|Il est joli, Sarah.
+copain|Il nage, presque.
 narrateur|Puis Nino reprend le chausson.
-papa|Tu as proposé court, juste assez.
+papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
       </c>
@@ -6031,12 +6031,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. La ficelle garde encore un peu de savon. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. La ficelle garde encore un peu de savon. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. La ficelle garde encore un peu de savon. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. La ficelle garde encore un peu de savon. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6172,14 +6172,14 @@
       <c r="AW29" t="inlineStr">
         <is>
           <t>narrateur|Le petit regard est déjà fini.
-copain|Le poisson a brillé, une fois.
-enfant-f|Merci d'avoir regardé.
-papa|Vous avez vu juste assez.
-maman|La mare entre, maintenant.
+copain|Il nageait, presque.
+enfant-f|Tu as vu, une seconde.
+papa|Un œil a suffi, déjà.
+maman|Le chausson est chaussé, maintenant.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Nino fait un signe vers le seau.
-enfant-f|On l'a vue, une minute.
-narrateur|Le radiateur reprend, tout doux.</t>
+narrateur|Nino s'assoit au bord du seau.
+enfant-f|On tire, tout doux.
+narrateur|Le radiateur reprend, tout bas.</t>
         </is>
       </c>
     </row>
@@ -6206,12 +6206,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le canapé garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le canapé garde sa rive, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le canapé garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le canapé garde sa rive, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6349,12 +6349,12 @@
           <t>enfant-f|On pêche plus tard, alors ?
 copain|Oui, plus tard.
 enfant-f|D'accord.
-narrateur|Le canapé garde sa place, tout calme.
+narrateur|Le canapé garde sa rive, tout calme.
 narrateur|Nino serre encore le chausson.
 copain|Garde un poisson pour moi.
-enfant-f|Il t'attend.
-papa|Tu as proposé une autre heure.
-maman|Il a dit oui, pour plus tard.</t>
+enfant-f|Il t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.</t>
         </is>
       </c>
     </row>
@@ -6381,12 +6381,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. La ficelle garde encore un peu de savon. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. La ficelle garde encore un peu de savon. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. La ficelle garde encore un peu de savon. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. La ficelle garde encore un peu de savon. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6523,11 +6523,11 @@
         <is>
           <t>narrateur|Nino enfile encore, un instant.
 enfant-f|Plus tard, il a dit.
-enfant-f|Le poisson t'attend.
-papa|Tu as proposé une autre heure.
-maman|Le seau attend, tout doux.
+enfant-f|Le poisson t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.
 narrateur|La ficelle garde encore un peu de savon.
-narrateur|Sarah garde une place, tout calme.
+narrateur|Sarah laisse un poisson à part.
 enfant-f|La mare t'attend, Nino.
 narrateur|La ficelle fait un pont, encore.</t>
         </is>
@@ -7293,12 +7293,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le seau près de la boîte. Nino tient encore la clé. Nino, le seau est bleu. Une note tinte, puis une autre. Ma chanson n'est pas finie. Tu viens à la table ? J'ai pas fini. Il reste dans sa chanson. Tu proposes comment, Sarah ?</t>
+          <t>Sarah pose le seau près de la boîte. Nino penche l'oreille, tout près. Nino, le seau est bleu. La clé glisse, puis reprend. Elle n'a pas dit au revoir. Tu viens à la table ? Cette chanson, d'abord. Il suit encore la note. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le seau près de la boîte. Nino tient encore la clé. Nino, le seau est bleu. Une note tinte, puis une autre. Ma chanson n'est pas finie. Tu viens à la table ? J'ai pas fini. Il reste dans sa chanson. Tu proposes comment, Sarah ?</t>
+          <t>Sarah pose le seau près de la boîte. Nino penche l'oreille, tout près. Nino, le seau est bleu. La clé glisse, puis reprend. Elle n'a pas dit au revoir. Tu viens à la table ? Cette chanson, d'abord. Il suit encore la note. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7434,14 +7434,14 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|Sarah pose le seau près de la boîte.
-narrateur|Nino tient encore la clé.
+narrateur|Nino penche l'oreille, tout près.
 enfant-f|Nino, le seau est bleu.
-narrateur|Une note tinte, puis une autre.
-copain|Ma chanson n'est pas finie.
+narrateur|La clé glisse, puis reprend.
+copain|Elle n'a pas dit au revoir.
 enfant-f|Tu viens à la table ?
-copain|J'ai pas fini.
-papa|Il reste dans sa chanson.
-maman|Tu proposes comment, Sarah ?</t>
+copain|Cette chanson, d'abord.
+papa|Il suit encore la note.
+maman|Tu restes près de lui ?</t>
         </is>
       </c>
     </row>
@@ -7660,12 +7660,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. Le seau bleu attend, sans bouger. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. Le seau bleu attend, sans bouger. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. Le seau bleu attend, sans bouger. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. Le seau bleu attend, sans bouger. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7800,15 +7800,15 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends un peu.
+          <t>enfant-f|J'attends la dernière note.
 copain|Merci, Sarah.
-narrateur|La boîte tourne sa dernière note.
+narrateur|Elle compte les tintes, sur ses doigts.
 narrateur|Le seau bleu attend, sans bouger.
-narrateur|Nino pose la clé, enfin.
-copain|Ma chanson est finie, maintenant.
+narrateur|La boîte s'arrête, pile.
+copain|Elle a dit au revoir.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé sa chanson finir.</t>
+copain|Oui, j'apporte la clé.
+papa|Tu as laissé la chanson finir.</t>
         </is>
       </c>
     </row>
@@ -7835,12 +7835,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. Le seau bleu garde un poisson plat. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. Le seau bleu garde un poisson plat. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. Le seau bleu garde un poisson plat. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. Le seau bleu garde un poisson plat. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7975,14 +7975,14 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Une nageoire jaune tremble dans le seau.
-copain|C'est une prise, Sarah ?
-enfant-f|Oui, elle est là.
-papa|Vous avez attendu le bon moment.
-maman|Le papier est encore un peu chaud.
+          <t>narrateur|La ficelle tremble, puis un papier vient.
+copain|Il a mordu, Sarah ?
+enfant-f|Oui, tout plat.
+papa|La chanson a laissé la place.
+maman|Le seau fait un petit ploc.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino souffle sur le poisson, tout petit.
-enfant-f|C'est notre mare, maintenant.
+narrateur|Nino pose la clé à côté du seau.
+enfant-f|La mare chante, maintenant.
 narrateur|Un peu de savon reste sur le papier.</t>
         </is>
       </c>
@@ -8010,12 +8010,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre la table. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre la table. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre la table. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre la table. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8150,15 +8150,15 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, je te propose la mare.
-narrateur|Elle parle tout contre la table.
+          <t>enfant-f|Nino, un poisson t'écoute.
+narrateur|Elle glisse un poisson contre la table.
 narrateur|Sa voix reste tout bas, près de lui.
-copain|J'ai entendu, Sarah.
-enfant-f|Tu peux dire non.
-copain|Oui, je viens.
-narrateur|Il ferme la boîte, tout doux.
-papa|Ta voix est restée tout bas.
-maman|Il a choisi de lui-même.</t>
+copain|Il a une oreille, lui aussi ?
+enfant-f|Oui, tout calme.
+copain|Je viens, alors.
+narrateur|Il pose la clé, sans la perdre.
+papa|Tu as parlé tout contre lui.
+maman|Il a dit oui, tout seul.</t>
         </is>
       </c>
     </row>
@@ -8185,12 +8185,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. Le seau bleu garde un poisson plat. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. Le seau bleu garde un poisson plat. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. Le seau bleu garde un poisson plat. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. Le seau bleu garde un poisson plat. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8325,14 +8325,14 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|La boîte est fermée, contre le genou.
-enfant-f|Tu as dit oui, tout bas.
-copain|J'avais entendu, près de toi.
-papa|Ta voix est restée tout bas.
-maman|Pêchez un peu, tout doux.
+          <t>narrateur|Le poisson collé écoute encore, un peu.
+enfant-f|Il t'a attendu, tout bas.
+copain|J'ai dit oui, près de toi.
+papa|Ta voix n'a pas cassé la note.
+maman|Pêchez, maintenant, tout doux.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino pose sa joue, tout calme.
-enfant-f|Reste autant que tu veux.
+narrateur|Nino tient le bâton, tout calme.
+enfant-f|On tire ensemble, tout lent.
 narrateur|La clé de la boîte dort, enfin.</t>
         </is>
       </c>
@@ -8360,12 +8360,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit près de la table. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit près de la table. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit près de la table. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit près de la table. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8503,12 +8503,12 @@
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit près de la table.
 narrateur|Elle ne touche pas la clé.
-copain|Tu écoutes, toi aussi ?
-enfant-f|Oui, avec toi.
-narrateur|Deux oreilles, maintenant, sur la boîte.
-copain|Après, on va pêcher.
-papa|Tu es restée près de lui.
-maman|Il a proposé la suite.</t>
+copain|Tu entends le ding, toi aussi ?
+enfant-f|Oui, dans le ventre.
+narrateur|Un dernier ding les fait sauter.
+copain|On pêche, après ça.
+papa|Tu as écouté sa boîte.
+maman|C'est lui qui a dit après.</t>
         </is>
       </c>
     </row>
@@ -8535,12 +8535,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. Le seau bleu garde un poisson plat. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. Le seau bleu garde un poisson plat. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. Le seau bleu garde un poisson plat. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. Le seau bleu garde un poisson plat. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8675,14 +8675,14 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Après la chanson, la ficelle descend.
-copain|On a écouté ensemble, d'abord.
-enfant-f|Puis tu as dit : on y va.
-maman|Deux oreilles, puis un poisson.
-papa|Le salon redevient calme.
+          <t>narrateur|Après le ding, la ficelle descend.
+copain|On a sauté, d'abord.
+enfant-f|Puis tu as dit : on pêche.
+maman|Un ding, puis un poisson.
+papa|Le salon redevient tiède.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino rit, tout petit.
-enfant-f|La mare t'a attendu.
+narrateur|Nino rit encore, tout petit.
+enfant-f|La mare a attendu le ding.
 narrateur|Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
@@ -8710,12 +8710,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Nino a déjà son camion, à la table. Le seau bleu attend, tout près. Nino, tu veux un poisson ? Mon camion n'est pas garé. On charge le seau ? Pas maintenant. Deux jeux, trop loin l'un de l'autre. Il n'a pas fini, Sarah. Tu proposes comment, alors ?</t>
+          <t>Nino a déjà son camion, à la table. Le seau bleu attend, tout près. Nino, tu veux un poisson ? Il va au garage, encore. On le met dans le seau ? Le garage, d'abord. Une roue frotte le bois, tout sec. Le camion n'est pas rentré. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Nino a déjà son camion, à la table. Le seau bleu attend, tout près. Nino, tu veux un poisson ? Mon camion n'est pas garé. On charge le seau ? Pas maintenant. Deux jeux, trop loin l'un de l'autre. Il n'a pas fini, Sarah. Tu proposes comment, alors ?</t>
+          <t>Nino a déjà son camion, à la table. Le seau bleu attend, tout près. Nino, tu veux un poisson ? Il va au garage, encore. On le met dans le seau ? Le garage, d'abord. Une roue frotte le bois, tout sec. Le camion n'est pas rentré. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8853,12 +8853,12 @@
           <t>narrateur|Nino a déjà son camion, à la table.
 narrateur|Le seau bleu attend, tout près.
 enfant-f|Nino, tu veux un poisson ?
-copain|Mon camion n'est pas garé.
-enfant-f|On charge le seau ?
-copain|Pas maintenant.
-narrateur|Deux jeux, trop loin l'un de l'autre.
-papa|Il n'a pas fini, Sarah.
-maman|Tu proposes comment, alors ?</t>
+copain|Il va au garage, encore.
+enfant-f|On le met dans le seau ?
+copain|Le garage, d'abord.
+narrateur|Une roue frotte le bois, tout sec.
+papa|Le camion n'est pas rentré.
+maman|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -9077,12 +9077,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le seau bleu garde son bois. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le seau bleu garde son bois. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le seau bleu garde son bois. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le seau bleu garde son bois. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9217,15 +9217,15 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends qu'il gare.
+          <t>enfant-f|J'attends le garage.
 copain|Merci, Sarah.
 narrateur|Le seau bleu garde son bois.
-narrateur|Le camion s'arrête, pile.
-copain|C'est garé, maintenant.
+narrateur|Le camion se glisse entre deux livres.
+copain|Il est rentré, maintenant.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé son camion finir.
-maman|Il a dit oui, à son heure.</t>
+copain|Oui, je laisse les roues.
+papa|Tu as laissé le garage finir.
+maman|Il a dit oui, après.</t>
         </is>
       </c>
     </row>
@@ -9252,12 +9252,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. Le seau bleu garde un poisson plat. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. Le seau bleu garde un poisson plat. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. Le seau bleu garde un poisson plat. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. Le seau bleu garde un poisson plat. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9392,14 +9392,14 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Le camion dort, près du seau.
-copain|J'ai fini, Sarah.
-enfant-f|Tu as dit oui.
-papa|Vous tenez tous les deux, maintenant.
-maman|Le poisson descend jusqu'à vous.
+          <t>narrateur|Le camion dort entre les livres.
+copain|Le garage est fermé, Sarah.
+enfant-f|Tu as dit oui, après.
+papa|Les roues se sont tues.
+maman|Le poisson glisse vers le seau.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino tape deux fois, tout doux.
-enfant-f|C'est le signal.
+narrateur|Nino souffle sur la nageoire, tout petit.
+enfant-f|Il nage, dans le bleu.
 narrateur|Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
@@ -9427,12 +9427,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sur la table. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur le bois. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sur la table. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur le bois. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9567,15 +9567,15 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un poisson dans le camion ?
-narrateur|Elle tend le poisson, sur la table.
-copain|Un tout petit, alors.
+          <t>enfant-f|Nino, un poisson voyageur ?
+narrateur|Elle pose le poisson sur le bois.
+copain|Il tient, sur le camion ?
+enfant-f|Tout plat, oui.
+narrateur|Le papier colle un peu, puis tient.
+copain|On va jusqu'au seau, alors.
 enfant-f|D'accord.
-narrateur|Le papier glisse, tout doux.
-copain|Il est tout plat, dedans.
-enfant-f|On est deux, maintenant.
-papa|Le poisson est resté dans sa main.
-maman|Il a pris ce qu'il voulait.</t>
+papa|Le poisson a pris la route.
+maman|Il a choisi le voyage.</t>
         </is>
       </c>
     </row>
@@ -9602,12 +9602,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. Le seau bleu garde un poisson plat. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. Le seau bleu garde un poisson plat. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. Le seau bleu garde un poisson plat. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. Le seau bleu garde un poisson plat. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9742,13 +9742,13 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le camion a un poisson, maintenant.
-enfant-f|Le tien, et le mien.
-copain|Il était plat, Sarah.
-papa|Vous avez partagé sans tout casser.
-maman|La mare, au fond, pour deux.
+          <t>narrateur|Le camion roule jusqu'au seau.
+enfant-f|Le voyageur descend, tout plat.
+copain|Il a tenu sur le capot.
+papa|Vous avez fait une route, ensemble.
+maman|Le seau devient un port, maintenant.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino souffle, puis Sarah souffle.
+narrateur|Nino pousse une dernière fois, tout doux.
 enfant-f|On reste encore un peu.
 narrateur|Un poisson plat dort sur le bois.</t>
         </is>
@@ -9777,12 +9777,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste sur la table. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste sur la table. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste sur la table. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste sur la table. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9919,13 +9919,13 @@
         <is>
           <t>copain|Pas de poisson, Sarah.
 enfant-f|D'accord.
-enfant-f|Je garde le seau, alors.
+enfant-f|Je pêche ici, alors.
 narrateur|Le seau reste sur la table.
-narrateur|Elle pêche de son côté, tout calme.
-copain|Tu peux parler, d'ici.
-enfant-f|Je reste près de toi.
+narrateur|Un poisson se colle à sa chaussette.
+copain|Il t'a pêchée, toi !
+enfant-f|Je ris, d'à côté.
 papa|Tu as gardé ton seau.
-maman|Vous êtes encore ensemble.</t>
+maman|Le camion est resté à lui.</t>
         </is>
       </c>
     </row>
@@ -9952,12 +9952,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. Le seau bleu garde un poisson plat. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. Le seau bleu garde un poisson plat. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. Le seau bleu garde un poisson plat. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. Le seau bleu garde un poisson plat. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10092,14 +10092,14 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Deux jeux restent côte à côte.
-copain|Tu n'as pas pris mon camion.
+          <t>narrateur|Le camion reste à sa place.
+copain|Tu n'as pas pris mes roues.
 enfant-f|Tu avais dit non.
-papa|Son camion est resté à lui.
-maman|Vous vous parlez encore, d'ici.
+papa|Son garage est resté à lui.
+maman|La chaussette a eu un poisson.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino tend une roue, alors.
-enfant-f|Je la prends, d'à côté.
+narrateur|Nino rit, puis pousse encore.
+enfant-f|Je pêche, tu roules.
 narrateur|Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
@@ -10127,12 +10127,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Nino quitte la table, un pied nu. J'ai un chausson, Sarah. Le seau est encore vide. Il ne s'assoit plus. Tu reviens au seau ? Quand j'ai mes chaussons, d'abord. Il cherche encore, tout tendu. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino quitte la table, un pied nu. J'ai un pied froid, Sarah. Le seau est encore vide. Le chausson droit est déjà chaud. Tu reviens au seau ? L'autre chausson, d'abord. Il cherche encore, tout tendu. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Nino quitte la table, un pied nu. J'ai un chausson, Sarah. Le seau est encore vide. Il ne s'assoit plus. Tu reviens au seau ? Quand j'ai mes chaussons, d'abord. Il cherche encore, tout tendu. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino quitte la table, un pied nu. J'ai un pied froid, Sarah. Le seau est encore vide. Le chausson droit est déjà chaud. Tu reviens au seau ? L'autre chausson, d'abord. Il cherche encore, tout tendu. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10268,14 +10268,14 @@
       <c r="AW52" t="inlineStr">
         <is>
           <t>narrateur|Nino quitte la table, un pied nu.
-copain|J'ai un chausson, Sarah.
+copain|J'ai un pied froid, Sarah.
 enfant-f|Le seau est encore vide.
-narrateur|Il ne s'assoit plus.
+narrateur|Le chausson droit est déjà chaud.
 enfant-f|Tu reviens au seau ?
-copain|Quand j'ai mes chaussons, d'abord.
+copain|L'autre chausson, d'abord.
 maman|Il cherche encore, tout tendu.
-papa|L'autre chausson n'est pas là.
-maman|Tu proposes comment, Sarah ?</t>
+papa|Le second n'est pas là.
+maman|Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
     </row>
@@ -10494,12 +10494,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche sous la table, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille sous la table, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche sous la table, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille sous la table, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10635,14 +10635,14 @@
       <c r="AW54" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle cherche sous la table, tout doux.
-narrateur|Le second chausson apparaît, enfin.
-copain|Tu l'as vu, toi aussi ?
-enfant-f|Oui, sous le bord.
+narrateur|Elle fouille sous la table, tout doux.
+narrateur|Un chausson chaud apparaît, enfin.
+copain|Il s'était caché !
+enfant-f|Près du bord, oui.
 narrateur|Deux pieds, maintenant, tout chauds.
-copain|Il était là !
-papa|Tu as aidé à son heure.
-maman|Vous l'avez eu, tous les deux.</t>
+copain|On peut pêcher, là.
+papa|Tu as cherché avec lui.
+maman|Le pied froid n'a plus froid.</t>
         </is>
       </c>
     </row>
@@ -10669,12 +10669,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. Le seau bleu garde un poisson plat. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. Le seau bleu garde un poisson plat. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. Le seau bleu garde un poisson plat. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. Le seau bleu garde un poisson plat. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10810,13 +10810,13 @@
       <c r="AW55" t="inlineStr">
         <is>
           <t>narrateur|Les deux chaussons sont chauds, enfin.
-copain|On l'a eu, ensemble.
-enfant-f|Puis la mare est arrivée.
-papa|Vous avez aidé à son heure.
+copain|Le pied froid n'a plus froid.
+enfant-f|On peut pêcher, là.
+papa|Vous avez cherché ensemble.
 maman|Le seau attend encore, tout doux.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino fait un signe vers le tapis.
-enfant-f|La mare t'a vu, une minute.
+narrateur|Nino s'allonge, le pied au chaud.
+enfant-f|La mare est tiède, pour deux.
 narrateur|Un fil jaune passe, tout loin.</t>
         </is>
       </c>
@@ -10844,12 +10844,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent le seau, une seconde. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers le seau, une seconde. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent le seau, une seconde. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers le seau, une seconde. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -10987,11 +10987,11 @@
           <t>enfant-f|Un tout petit regard, Nino ?
 copain|Très petit, alors.
 enfant-f|D'accord.
-narrateur|Ils regardent le seau, une seconde.
+narrateur|Ils se penchent vers le seau, une seconde.
 narrateur|Un poisson jaune brille, une seconde.
-copain|Il est joli, Sarah.
+copain|Il nage, presque.
 narrateur|Puis Nino reprend le chausson.
-papa|Tu as proposé court, juste assez.
+papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
       </c>
@@ -11019,12 +11019,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. Le seau bleu garde un poisson plat. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. Le seau bleu garde un poisson plat. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. Le seau bleu garde un poisson plat. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. Le seau bleu garde un poisson plat. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11160,14 +11160,14 @@
       <c r="AW57" t="inlineStr">
         <is>
           <t>narrateur|Le petit regard est déjà fini.
-copain|Le poisson a brillé, une fois.
-enfant-f|Merci d'avoir regardé.
-papa|Vous avez vu juste assez.
-maman|La mare entre, maintenant.
+copain|Il nageait, presque.
+enfant-f|Tu as vu, une seconde.
+papa|Un œil a suffi, déjà.
+maman|Le chausson est chaussé, maintenant.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Nino fait un signe vers le seau.
-enfant-f|On l'a vue, une minute.
-narrateur|Le radiateur reprend, tout doux.</t>
+narrateur|Nino s'assoit au bord du seau.
+enfant-f|On tire, tout doux.
+narrateur|Le radiateur reprend, tout bas.</t>
         </is>
       </c>
     </row>
@@ -11194,12 +11194,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. La table garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. La table garde le seau, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. La table garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. La table garde le seau, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11337,12 +11337,12 @@
           <t>enfant-f|On pêche plus tard, alors ?
 copain|Oui, plus tard.
 enfant-f|D'accord.
-narrateur|La table garde sa place, tout calme.
+narrateur|La table garde le seau, tout calme.
 narrateur|Nino serre encore le chausson.
 copain|Garde un poisson pour moi.
-enfant-f|Il t'attend.
-papa|Tu as proposé une autre heure.
-maman|Il a dit oui, pour plus tard.</t>
+enfant-f|Il t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.</t>
         </is>
       </c>
     </row>
@@ -11369,12 +11369,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. Le seau bleu garde un poisson plat. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. Le seau bleu garde un poisson plat. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. Le seau bleu garde un poisson plat. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. Le seau bleu garde un poisson plat. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11511,11 +11511,11 @@
         <is>
           <t>narrateur|Nino enfile encore, un instant.
 enfant-f|Plus tard, il a dit.
-enfant-f|Le poisson t'attend.
-papa|Tu as proposé une autre heure.
-maman|Le seau attend, tout doux.
+enfant-f|Le poisson t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.
 narrateur|Le seau bleu garde un poisson plat.
-narrateur|Sarah garde une place, tout calme.
+narrateur|Sarah laisse un poisson à part.
 enfant-f|La mare t'attend, Nino.
 narrateur|La ficelle fait un pont, encore.</t>
         </is>
@@ -12281,12 +12281,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le poisson jaune tremble près du tapis. Nino tourne la clé, tout bas. Nino, ma mare est tiède. Le radiateur chante avec la boîte. Ma chanson n'est pas finie. Tu viens t'allonger ? J'ai pas fini. La boîte tient encore sa note. Tu proposes comment, Sarah ?</t>
+          <t>Le poisson jaune tremble près du tapis. Nino tourne la clé, tout bas. Nino, ma mare est tiède. Le radiateur chante avec la boîte. Elle n'a pas dit au revoir. Tu viens t'allonger ? Cette chanson, d'abord. La note n'est pas partie. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Le poisson jaune tremble près du tapis. Nino tourne la clé, tout bas. Nino, ma mare est tiède. Le radiateur chante avec la boîte. Ma chanson n'est pas finie. Tu viens t'allonger ? J'ai pas fini. La boîte tient encore sa note. Tu proposes comment, Sarah ?</t>
+          <t>Le poisson jaune tremble près du tapis. Nino tourne la clé, tout bas. Nino, ma mare est tiède. Le radiateur chante avec la boîte. Elle n'a pas dit au revoir. Tu viens t'allonger ? Cette chanson, d'abord. La note n'est pas partie. Tu restes près de lui ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12425,11 +12425,11 @@
 narrateur|Nino tourne la clé, tout bas.
 enfant-f|Nino, ma mare est tiède.
 narrateur|Le radiateur chante avec la boîte.
-copain|Ma chanson n'est pas finie.
+copain|Elle n'a pas dit au revoir.
 enfant-f|Tu viens t'allonger ?
-copain|J'ai pas fini.
-maman|La boîte tient encore sa note.
-papa|Tu proposes comment, Sarah ?</t>
+copain|Cette chanson, d'abord.
+maman|La note n'est pas partie.
+papa|Tu restes près de lui ?</t>
         </is>
       </c>
     </row>
@@ -12648,12 +12648,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. Le poisson jaune attend, tout plat. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. Le poisson jaune attend, tout plat. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>J'attends un peu. Merci, Sarah. La boîte tourne sa dernière note. Le poisson jaune attend, tout plat. Nino pose la clé, enfin. Ma chanson est finie, maintenant. Tu viens, alors ? Oui. Tu as laissé sa chanson finir.</t>
+          <t>J'attends la dernière note. Merci, Sarah. Elle compte les tintes, sur ses doigts. Le poisson jaune attend, tout plat. La boîte s'arrête, pile. Elle a dit au revoir. Tu viens, alors ? Oui, j'apporte la clé. Tu as laissé la chanson finir.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12788,15 +12788,15 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends un peu.
+          <t>enfant-f|J'attends la dernière note.
 copain|Merci, Sarah.
-narrateur|La boîte tourne sa dernière note.
+narrateur|Elle compte les tintes, sur ses doigts.
 narrateur|Le poisson jaune attend, tout plat.
-narrateur|Nino pose la clé, enfin.
-copain|Ma chanson est finie, maintenant.
+narrateur|La boîte s'arrête, pile.
+copain|Elle a dit au revoir.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé sa chanson finir.</t>
+copain|Oui, j'apporte la clé.
+papa|Tu as laissé la chanson finir.</t>
         </is>
       </c>
     </row>
@@ -12823,12 +12823,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. Le tapis garde un fil, tout calme. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. Le tapis garde un fil, tout calme. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Une nageoire jaune tremble dans le seau. C'est une prise, Sarah ? Oui, elle est là. Vous avez attendu le bon moment. Le papier est encore un peu chaud. Le tapis garde un fil, tout calme. Nino souffle sur le poisson, tout petit. C'est notre mare, maintenant. Un peu de savon reste sur le papier.</t>
+          <t>La ficelle tremble, puis un papier vient. Il a mordu, Sarah ? Oui, tout plat. La chanson a laissé la place. Le seau fait un petit ploc. Le tapis garde un fil, tout calme. Nino pose la clé à côté du seau. La mare chante, maintenant. Un peu de savon reste sur le papier.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12963,14 +12963,14 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Une nageoire jaune tremble dans le seau.
-copain|C'est une prise, Sarah ?
-enfant-f|Oui, elle est là.
-papa|Vous avez attendu le bon moment.
-maman|Le papier est encore un peu chaud.
+          <t>narrateur|La ficelle tremble, puis un papier vient.
+copain|Il a mordu, Sarah ?
+enfant-f|Oui, tout plat.
+papa|La chanson a laissé la place.
+maman|Le seau fait un petit ploc.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino souffle sur le poisson, tout petit.
-enfant-f|C'est notre mare, maintenant.
+narrateur|Nino pose la clé à côté du seau.
+enfant-f|La mare chante, maintenant.
 narrateur|Un peu de savon reste sur le papier.</t>
         </is>
       </c>
@@ -12998,12 +12998,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre le tapis. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre le tapis. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Nino, je te propose la mare. Elle parle tout contre le tapis. Sa voix reste tout bas, près de lui. J'ai entendu, Sarah. Tu peux dire non. Oui, je viens. Il ferme la boîte, tout doux. Ta voix est restée tout bas. Il a choisi de lui-même.</t>
+          <t>Nino, un poisson t'écoute. Elle glisse un poisson contre le tapis. Sa voix reste tout bas, près de lui. Il a une oreille, lui aussi ? Oui, tout calme. Je viens, alors. Il pose la clé, sans la perdre. Tu as parlé tout contre lui. Il a dit oui, tout seul.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13138,15 +13138,15 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, je te propose la mare.
-narrateur|Elle parle tout contre le tapis.
+          <t>enfant-f|Nino, un poisson t'écoute.
+narrateur|Elle glisse un poisson contre le tapis.
 narrateur|Sa voix reste tout bas, près de lui.
-copain|J'ai entendu, Sarah.
-enfant-f|Tu peux dire non.
-copain|Oui, je viens.
-narrateur|Il ferme la boîte, tout doux.
-papa|Ta voix est restée tout bas.
-maman|Il a choisi de lui-même.</t>
+copain|Il a une oreille, lui aussi ?
+enfant-f|Oui, tout calme.
+copain|Je viens, alors.
+narrateur|Il pose la clé, sans la perdre.
+papa|Tu as parlé tout contre lui.
+maman|Il a dit oui, tout seul.</t>
         </is>
       </c>
     </row>
@@ -13173,12 +13173,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. Le tapis garde un fil, tout calme. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. Le tapis garde un fil, tout calme. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>La boîte est fermée, contre le genou. Tu as dit oui, tout bas. J'avais entendu, près de toi. Ta voix est restée tout bas. Pêchez un peu, tout doux. Le tapis garde un fil, tout calme. Nino pose sa joue, tout calme. Reste autant que tu veux. La clé de la boîte dort, enfin.</t>
+          <t>Le poisson collé écoute encore, un peu. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, tout doux. Le tapis garde un fil, tout calme. Nino tient le bâton, tout calme. On tire ensemble, tout lent. La clé de la boîte dort, enfin.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13313,14 +13313,14 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|La boîte est fermée, contre le genou.
-enfant-f|Tu as dit oui, tout bas.
-copain|J'avais entendu, près de toi.
-papa|Ta voix est restée tout bas.
-maman|Pêchez un peu, tout doux.
+          <t>narrateur|Le poisson collé écoute encore, un peu.
+enfant-f|Il t'a attendu, tout bas.
+copain|J'ai dit oui, près de toi.
+papa|Ta voix n'a pas cassé la note.
+maman|Pêchez, maintenant, tout doux.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino pose sa joue, tout calme.
-enfant-f|Reste autant que tu veux.
+narrateur|Nino tient le bâton, tout calme.
+enfant-f|On tire ensemble, tout lent.
 narrateur|La clé de la boîte dort, enfin.</t>
         </is>
       </c>
@@ -13348,12 +13348,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit près du radiateur. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit près du radiateur. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit près du radiateur. Elle ne touche pas la clé. Tu écoutes, toi aussi ? Oui, avec toi. Deux oreilles, maintenant, sur la boîte. Après, on va pêcher. Tu es restée près de lui. Il a proposé la suite.</t>
+          <t>Je m'assois à côté. Sarah s'assoit près du radiateur. Elle ne touche pas la clé. Tu entends le ding, toi aussi ? Oui, dans le ventre. Un dernier ding les fait sauter. On pêche, après ça. Tu as écouté sa boîte. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13491,12 +13491,12 @@
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit près du radiateur.
 narrateur|Elle ne touche pas la clé.
-copain|Tu écoutes, toi aussi ?
-enfant-f|Oui, avec toi.
-narrateur|Deux oreilles, maintenant, sur la boîte.
-copain|Après, on va pêcher.
-papa|Tu es restée près de lui.
-maman|Il a proposé la suite.</t>
+copain|Tu entends le ding, toi aussi ?
+enfant-f|Oui, dans le ventre.
+narrateur|Un dernier ding les fait sauter.
+copain|On pêche, après ça.
+papa|Tu as écouté sa boîte.
+maman|C'est lui qui a dit après.</t>
         </is>
       </c>
     </row>
@@ -13523,12 +13523,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. Le tapis garde un fil, tout calme. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. Le tapis garde un fil, tout calme. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Après la chanson, la ficelle descend. On a écouté ensemble, d'abord. Puis tu as dit : on y va. Deux oreilles, puis un poisson. Le salon redevient calme. Le tapis garde un fil, tout calme. Nino rit, tout petit. La mare t'a attendu. Deux mains tiennent le bâton, déjà.</t>
+          <t>Après le ding, la ficelle descend. On a sauté, d'abord. Puis tu as dit : on pêche. Un ding, puis un poisson. Le salon redevient tiède. Le tapis garde un fil, tout calme. Nino rit encore, tout petit. La mare a attendu le ding. Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13663,14 +13663,14 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Après la chanson, la ficelle descend.
-copain|On a écouté ensemble, d'abord.
-enfant-f|Puis tu as dit : on y va.
-maman|Deux oreilles, puis un poisson.
-papa|Le salon redevient calme.
+          <t>narrateur|Après le ding, la ficelle descend.
+copain|On a sauté, d'abord.
+enfant-f|Puis tu as dit : on pêche.
+maman|Un ding, puis un poisson.
+papa|Le salon redevient tiède.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino rit, tout petit.
-enfant-f|La mare t'a attendu.
+narrateur|Nino rit encore, tout petit.
+enfant-f|La mare a attendu le ding.
 narrateur|Deux mains tiennent le bâton, déjà.</t>
         </is>
       </c>
@@ -13698,12 +13698,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Nino pousse le camion sur le tapis. Une roue passe sur la ficelle. Nino, la mare est tiède. Mon camion n'est pas garé. Tu t'allonges avec moi ? Après, peut-être. Le poisson tremble, tout plat. Il conduit encore, tout concentré. Tu proposes comment, Sarah ?</t>
+          <t>Nino pousse le camion sur le tapis. Une roue passe sur la ficelle. Nino, la mare est tiède. Il va au garage, encore. Tu t'allonges avec moi ? Le garage, d'abord. Le poisson tremble, tout plat. Il cherche encore sa place. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Nino pousse le camion sur le tapis. Une roue passe sur la ficelle. Nino, la mare est tiède. Mon camion n'est pas garé. Tu t'allonges avec moi ? Après, peut-être. Le poisson tremble, tout plat. Il conduit encore, tout concentré. Tu proposes comment, Sarah ?</t>
+          <t>Nino pousse le camion sur le tapis. Une roue passe sur la ficelle. Nino, la mare est tiède. Il va au garage, encore. Tu t'allonges avec moi ? Le garage, d'abord. Le poisson tremble, tout plat. Il cherche encore sa place. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13841,12 +13841,12 @@
           <t>narrateur|Nino pousse le camion sur le tapis.
 narrateur|Une roue passe sur la ficelle.
 enfant-f|Nino, la mare est tiède.
-copain|Mon camion n'est pas garé.
+copain|Il va au garage, encore.
 enfant-f|Tu t'allonges avec moi ?
-copain|Après, peut-être.
+copain|Le garage, d'abord.
 narrateur|Le poisson tremble, tout plat.
-maman|Il conduit encore, tout concentré.
-papa|Tu proposes comment, Sarah ?</t>
+maman|Il cherche encore sa place.
+papa|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -14065,12 +14065,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le poisson jaune garde le tapis. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le poisson jaune garde le tapis. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>J'attends qu'il gare. Merci, Sarah. Le poisson jaune garde le tapis. Le camion s'arrête, pile. C'est garé, maintenant. Tu viens, alors ? Oui. Tu as laissé son camion finir. Il a dit oui, à son heure.</t>
+          <t>J'attends le garage. Merci, Sarah. Le poisson jaune garde le tapis. Le camion se glisse entre deux livres. Il est rentré, maintenant. Tu viens, alors ? Oui, je laisse les roues. Tu as laissé le garage finir. Il a dit oui, après.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14205,15 +14205,15 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>enfant-f|J'attends qu'il gare.
+          <t>enfant-f|J'attends le garage.
 copain|Merci, Sarah.
 narrateur|Le poisson jaune garde le tapis.
-narrateur|Le camion s'arrête, pile.
-copain|C'est garé, maintenant.
+narrateur|Le camion se glisse entre deux livres.
+copain|Il est rentré, maintenant.
 enfant-f|Tu viens, alors ?
-copain|Oui.
-papa|Tu as laissé son camion finir.
-maman|Il a dit oui, à son heure.</t>
+copain|Oui, je laisse les roues.
+papa|Tu as laissé le garage finir.
+maman|Il a dit oui, après.</t>
         </is>
       </c>
     </row>
@@ -14240,12 +14240,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. Le tapis garde un fil, tout calme. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. Le tapis garde un fil, tout calme. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Le camion dort, près du seau. J'ai fini, Sarah. Tu as dit oui. Vous tenez tous les deux, maintenant. Le poisson descend jusqu'à vous. Le tapis garde un fil, tout calme. Nino tape deux fois, tout doux. C'est le signal. Une roue jaune sent encore le tapis.</t>
+          <t>Le camion dort entre les livres. Le garage est fermé, Sarah. Tu as dit oui, après. Les roues se sont tues. Le poisson glisse vers le seau. Le tapis garde un fil, tout calme. Nino souffle sur la nageoire, tout petit. Il nage, dans le bleu. Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14380,14 +14380,14 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Le camion dort, près du seau.
-copain|J'ai fini, Sarah.
-enfant-f|Tu as dit oui.
-papa|Vous tenez tous les deux, maintenant.
-maman|Le poisson descend jusqu'à vous.
+          <t>narrateur|Le camion dort entre les livres.
+copain|Le garage est fermé, Sarah.
+enfant-f|Tu as dit oui, après.
+papa|Les roues se sont tues.
+maman|Le poisson glisse vers le seau.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino tape deux fois, tout doux.
-enfant-f|C'est le signal.
+narrateur|Nino souffle sur la nageoire, tout petit.
+enfant-f|Il nage, dans le bleu.
 narrateur|Une roue jaune sent encore le tapis.</t>
         </is>
       </c>
@@ -14415,12 +14415,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sur le tapis. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur une roue. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Nino, un poisson dans le camion ? Elle tend le poisson, sur le tapis. Un tout petit, alors. D'accord. Le papier glisse, tout doux. Il est tout plat, dedans. On est deux, maintenant. Le poisson est resté dans sa main. Il a pris ce qu'il voulait.</t>
+          <t>Nino, un poisson voyageur ? Elle pose le poisson sur une roue. Il tient, sur le camion ? Tout plat, oui. Le papier colle un peu, puis tient. On va jusqu'au seau, alors. D'accord. Le poisson a pris la route. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14555,15 +14555,15 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un poisson dans le camion ?
-narrateur|Elle tend le poisson, sur le tapis.
-copain|Un tout petit, alors.
+          <t>enfant-f|Nino, un poisson voyageur ?
+narrateur|Elle pose le poisson sur une roue.
+copain|Il tient, sur le camion ?
+enfant-f|Tout plat, oui.
+narrateur|Le papier colle un peu, puis tient.
+copain|On va jusqu'au seau, alors.
 enfant-f|D'accord.
-narrateur|Le papier glisse, tout doux.
-copain|Il est tout plat, dedans.
-enfant-f|On est deux, maintenant.
-papa|Le poisson est resté dans sa main.
-maman|Il a pris ce qu'il voulait.</t>
+papa|Le poisson a pris la route.
+maman|Il a choisi le voyage.</t>
         </is>
       </c>
     </row>
@@ -14590,12 +14590,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. Le tapis garde un fil, tout calme. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. Le tapis garde un fil, tout calme. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le camion a un poisson, maintenant. Le tien, et le mien. Il était plat, Sarah. Vous avez partagé sans tout casser. La mare, au fond, pour deux. Le tapis garde un fil, tout calme. Nino souffle, puis Sarah souffle. On reste encore un peu. Un poisson plat dort sur le bois.</t>
+          <t>Le camion roule jusqu'au seau. Le voyageur descend, tout plat. Il a tenu sur le capot. Vous avez fait une route, ensemble. Le seau devient un port, maintenant. Le tapis garde un fil, tout calme. Nino pousse une dernière fois, tout doux. On reste encore un peu. Un poisson plat dort sur le bois.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14730,13 +14730,13 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le camion a un poisson, maintenant.
-enfant-f|Le tien, et le mien.
-copain|Il était plat, Sarah.
-papa|Vous avez partagé sans tout casser.
-maman|La mare, au fond, pour deux.
+          <t>narrateur|Le camion roule jusqu'au seau.
+enfant-f|Le voyageur descend, tout plat.
+copain|Il a tenu sur le capot.
+papa|Vous avez fait une route, ensemble.
+maman|Le seau devient un port, maintenant.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino souffle, puis Sarah souffle.
+narrateur|Nino pousse une dernière fois, tout doux.
 enfant-f|On reste encore un peu.
 narrateur|Un poisson plat dort sur le bois.</t>
         </is>
@@ -14765,12 +14765,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste près du radiateur. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste près du radiateur. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Pas de poisson, Sarah. D'accord. Je garde le seau, alors. Le seau reste près du radiateur. Elle pêche de son côté, tout calme. Tu peux parler, d'ici. Je reste près de toi. Tu as gardé ton seau. Vous êtes encore ensemble.</t>
+          <t>Pas de poisson, Sarah. D'accord. Je pêche ici, alors. Le seau reste près du radiateur. Un poisson se colle à sa chaussette. Il t'a pêchée, toi ! Je ris, d'à côté. Tu as gardé ton seau. Le camion est resté à lui.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14907,13 +14907,13 @@
         <is>
           <t>copain|Pas de poisson, Sarah.
 enfant-f|D'accord.
-enfant-f|Je garde le seau, alors.
+enfant-f|Je pêche ici, alors.
 narrateur|Le seau reste près du radiateur.
-narrateur|Elle pêche de son côté, tout calme.
-copain|Tu peux parler, d'ici.
-enfant-f|Je reste près de toi.
+narrateur|Un poisson se colle à sa chaussette.
+copain|Il t'a pêchée, toi !
+enfant-f|Je ris, d'à côté.
 papa|Tu as gardé ton seau.
-maman|Vous êtes encore ensemble.</t>
+maman|Le camion est resté à lui.</t>
         </is>
       </c>
     </row>
@@ -14940,12 +14940,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. Le tapis garde un fil, tout calme. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. Le tapis garde un fil, tout calme. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Deux jeux restent côte à côte. Tu n'as pas pris mon camion. Tu avais dit non. Son camion est resté à lui. Vous vous parlez encore, d'ici. Le tapis garde un fil, tout calme. Nino tend une roue, alors. Je la prends, d'à côté. Deux jeux se parlent, tout calme.</t>
+          <t>Le camion reste à sa place. Tu n'as pas pris mes roues. Tu avais dit non. Son garage est resté à lui. La chaussette a eu un poisson. Le tapis garde un fil, tout calme. Nino rit, puis pousse encore. Je pêche, tu roules. Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15080,14 +15080,14 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Deux jeux restent côte à côte.
-copain|Tu n'as pas pris mon camion.
+          <t>narrateur|Le camion reste à sa place.
+copain|Tu n'as pas pris mes roues.
 enfant-f|Tu avais dit non.
-papa|Son camion est resté à lui.
-maman|Vous vous parlez encore, d'ici.
+papa|Son garage est resté à lui.
+maman|La chaussette a eu un poisson.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino tend une roue, alors.
-enfant-f|Je la prends, d'à côté.
+narrateur|Nino rit, puis pousse encore.
+enfant-f|Je pêche, tu roules.
 narrateur|Deux jeux se parlent, tout calme.</t>
         </is>
       </c>
@@ -15115,12 +15115,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Nino se tient près du radiateur. J'ai un chausson, Sarah. Ma mare est déjà tiède. Il serre le chausson, tout calme. Tu t'allonges avec moi ? Quand j'ai mes chaussons, d'abord. Il cherche encore, tout près. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino se tient près du radiateur. J'ai un pied froid, Sarah. Ma mare est déjà tiède. Il serre un chausson, tout calme. Tu t'allonges avec moi ? L'autre chausson, d'abord. Il cherche encore, tout près. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Nino se tient près du radiateur. J'ai un chausson, Sarah. Ma mare est déjà tiède. Il serre le chausson, tout calme. Tu t'allonges avec moi ? Quand j'ai mes chaussons, d'abord. Il cherche encore, tout près. L'autre chausson n'est pas là. Tu proposes comment, Sarah ?</t>
+          <t>Nino se tient près du radiateur. J'ai un pied froid, Sarah. Ma mare est déjà tiède. Il serre un chausson, tout calme. Tu t'allonges avec moi ? L'autre chausson, d'abord. Il cherche encore, tout près. Le second n'est pas là. Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15256,14 +15256,14 @@
       <c r="AW80" t="inlineStr">
         <is>
           <t>narrateur|Nino se tient près du radiateur.
-copain|J'ai un chausson, Sarah.
+copain|J'ai un pied froid, Sarah.
 enfant-f|Ma mare est déjà tiède.
-narrateur|Il serre le chausson, tout calme.
+narrateur|Il serre un chausson, tout calme.
 enfant-f|Tu t'allonges avec moi ?
-copain|Quand j'ai mes chaussons, d'abord.
+copain|L'autre chausson, d'abord.
 papa|Il cherche encore, tout près.
-maman|L'autre chausson n'est pas là.
-papa|Tu proposes comment, Sarah ?</t>
+maman|Le second n'est pas là.
+papa|Tu l'aides, ou tu attends ?</t>
         </is>
       </c>
     </row>
@@ -15482,12 +15482,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche près du radiateur, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille près du radiateur, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle cherche près du radiateur, tout doux. Le second chausson apparaît, enfin. Tu l'as vu, toi aussi ? Oui, sous le bord. Deux pieds, maintenant, tout chauds. Il était là ! Tu as aidé à son heure. Vous l'avez eu, tous les deux.</t>
+          <t>J'aide un peu. Elle fouille près du radiateur, tout doux. Un chausson chaud apparaît, enfin. Il s'était caché ! Près du bord, oui. Deux pieds, maintenant, tout chauds. On peut pêcher, là. Tu as cherché avec lui. Le pied froid n'a plus froid.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15623,14 +15623,14 @@
       <c r="AW82" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle cherche près du radiateur, tout doux.
-narrateur|Le second chausson apparaît, enfin.
-copain|Tu l'as vu, toi aussi ?
-enfant-f|Oui, sous le bord.
+narrateur|Elle fouille près du radiateur, tout doux.
+narrateur|Un chausson chaud apparaît, enfin.
+copain|Il s'était caché !
+enfant-f|Près du bord, oui.
 narrateur|Deux pieds, maintenant, tout chauds.
-copain|Il était là !
-papa|Tu as aidé à son heure.
-maman|Vous l'avez eu, tous les deux.</t>
+copain|On peut pêcher, là.
+papa|Tu as cherché avec lui.
+maman|Le pied froid n'a plus froid.</t>
         </is>
       </c>
     </row>
@@ -15657,12 +15657,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. Le tapis garde un fil, tout calme. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. Le tapis garde un fil, tout calme. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Les deux chaussons sont chauds, enfin. On l'a eu, ensemble. Puis la mare est arrivée. Vous avez aidé à son heure. Le seau attend encore, tout doux. Le tapis garde un fil, tout calme. Nino fait un signe vers le tapis. La mare t'a vu, une minute. Un fil jaune passe, tout loin.</t>
+          <t>Les deux chaussons sont chauds, enfin. Le pied froid n'a plus froid. On peut pêcher, là. Vous avez cherché ensemble. Le seau attend encore, tout doux. Le tapis garde un fil, tout calme. Nino s'allonge, le pied au chaud. La mare est tiède, pour deux. Un fil jaune passe, tout loin.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15798,13 +15798,13 @@
       <c r="AW83" t="inlineStr">
         <is>
           <t>narrateur|Les deux chaussons sont chauds, enfin.
-copain|On l'a eu, ensemble.
-enfant-f|Puis la mare est arrivée.
-papa|Vous avez aidé à son heure.
+copain|Le pied froid n'a plus froid.
+enfant-f|On peut pêcher, là.
+papa|Vous avez cherché ensemble.
 maman|Le seau attend encore, tout doux.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino fait un signe vers le tapis.
-enfant-f|La mare t'a vu, une minute.
+narrateur|Nino s'allonge, le pied au chaud.
+enfant-f|La mare est tiède, pour deux.
 narrateur|Un fil jaune passe, tout loin.</t>
         </is>
       </c>
@@ -15832,12 +15832,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent la mare du tapis. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers la mare du tapis. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils regardent la mare du tapis. Un poisson jaune brille, une seconde. Il est joli, Sarah. Puis Nino reprend le chausson. Tu as proposé court, juste assez. Il a vu, puis choisi.</t>
+          <t>Un tout petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers la mare du tapis. Un poisson jaune brille, une seconde. Il nage, presque. Puis Nino reprend le chausson. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15975,11 +15975,11 @@
           <t>enfant-f|Un tout petit regard, Nino ?
 copain|Très petit, alors.
 enfant-f|D'accord.
-narrateur|Ils regardent la mare du tapis.
+narrateur|Ils se penchent vers la mare du tapis.
 narrateur|Un poisson jaune brille, une seconde.
-copain|Il est joli, Sarah.
+copain|Il nage, presque.
 narrateur|Puis Nino reprend le chausson.
-papa|Tu as proposé court, juste assez.
+papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
       </c>
@@ -16007,12 +16007,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. Le tapis garde un fil, tout calme. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. Le tapis garde un fil, tout calme. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Le petit regard est déjà fini. Le poisson a brillé, une fois. Merci d'avoir regardé. Vous avez vu juste assez. La mare entre, maintenant. Le tapis garde un fil, tout calme. Nino fait un signe vers le seau. On l'a vue, une minute. Le radiateur reprend, tout doux.</t>
+          <t>Le petit regard est déjà fini. Il nageait, presque. Tu as vu, une seconde. Un œil a suffi, déjà. Le chausson est chaussé, maintenant. Le tapis garde un fil, tout calme. Nino s'assoit au bord du seau. On tire, tout doux. Le radiateur reprend, tout bas.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16148,14 +16148,14 @@
       <c r="AW85" t="inlineStr">
         <is>
           <t>narrateur|Le petit regard est déjà fini.
-copain|Le poisson a brillé, une fois.
-enfant-f|Merci d'avoir regardé.
-papa|Vous avez vu juste assez.
-maman|La mare entre, maintenant.
+copain|Il nageait, presque.
+enfant-f|Tu as vu, une seconde.
+papa|Un œil a suffi, déjà.
+maman|Le chausson est chaussé, maintenant.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Nino fait un signe vers le seau.
-enfant-f|On l'a vue, une minute.
-narrateur|Le radiateur reprend, tout doux.</t>
+narrateur|Nino s'assoit au bord du seau.
+enfant-f|On tire, tout doux.
+narrateur|Le radiateur reprend, tout bas.</t>
         </is>
       </c>
     </row>
@@ -16182,12 +16182,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le tapis garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le tapis garde sa mare, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le tapis garde sa place, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend. Tu as proposé une autre heure. Il a dit oui, pour plus tard.</t>
+          <t>On pêche plus tard, alors ? Oui, plus tard. D'accord. Le tapis garde sa mare, tout calme. Nino serre encore le chausson. Garde un poisson pour moi. Il t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16325,12 +16325,12 @@
           <t>enfant-f|On pêche plus tard, alors ?
 copain|Oui, plus tard.
 enfant-f|D'accord.
-narrateur|Le tapis garde sa place, tout calme.
+narrateur|Le tapis garde sa mare, tout calme.
 narrateur|Nino serre encore le chausson.
 copain|Garde un poisson pour moi.
-enfant-f|Il t'attend.
-papa|Tu as proposé une autre heure.
-maman|Il a dit oui, pour plus tard.</t>
+enfant-f|Il t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.</t>
         </is>
       </c>
     </row>
@@ -16357,12 +16357,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. Le tapis garde un fil, tout calme. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. Le tapis garde un fil, tout calme. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend. Tu as proposé une autre heure. Le seau attend, tout doux. Le tapis garde un fil, tout calme. Sarah garde une place, tout calme. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
+          <t>Nino enfile encore, un instant. Plus tard, il a dit. Le poisson t'attend dans le seau. Tu as dit une autre heure. Le pied froid cherche encore. Le tapis garde un fil, tout calme. Sarah laisse un poisson à part. La mare t'attend, Nino. La ficelle fait un pont, encore.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16499,11 +16499,11 @@
         <is>
           <t>narrateur|Nino enfile encore, un instant.
 enfant-f|Plus tard, il a dit.
-enfant-f|Le poisson t'attend.
-papa|Tu as proposé une autre heure.
-maman|Le seau attend, tout doux.
+enfant-f|Le poisson t'attend dans le seau.
+papa|Tu as dit une autre heure.
+maman|Le pied froid cherche encore.
 narrateur|Le tapis garde un fil, tout calme.
-narrateur|Sarah garde une place, tout calme.
+narrateur|Sarah laisse un poisson à part.
 enfant-f|La mare t'attend, Nino.
 narrateur|La ficelle fait un pont, encore.</t>
         </is>
@@ -16526,7 +16526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16569,6 +16569,20 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-DIF-049 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-049.xlsx
+++ b/stories/arbres/TREE-DIF-049.xlsx
@@ -3276,17 +3276,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le poisson collé écoute un peu, encore. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.</t>
+          <t>Le poisson collé au canapé écoute, sans bouger. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;poisson&lt;/emphasis&gt; collé écoute un peu, encore. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;poisson&lt;/emphasis&gt; collé au canapé écoute, sans bouger. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;poisson&lt;/emphasis&gt; collé écoute un peu, encore. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;poisson&lt;/emphasis&gt; collé au canapé écoute, sans bouger. Il t'a attendu, tout bas. J'ai dit oui, près de toi. Ta voix n'a pas cassé la note. Pêchez, maintenant, sans crier. Nino tient le bâton, très calme. On tire ensemble, tout lent. La clé de la boîte dort contre le canapé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Le poisson collé écoute un peu, encore.
+          <t>narrateur|Le poisson collé au canapé écoute, sans bouger.
 enfant-f|Il t'a attendu, tout bas.
 copain|J'ai dit oui, près de toi.
 papa|Ta voix n'a pas cassé la note.
@@ -17304,7 +17304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17368,6 +17368,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>